<commit_message>
feat(magazine): bulk re-migrate remaining articles to two-column layout
Re-migrate arctic-surfing, san-diego-surf, ski-touring, and western-australia
to the same two-column aside layout as guide-la-skateparks (article left,
author byline + "Share This Story" rail), replacing the flattened version.

- generalize the magazine-article importer: match the author byline by the
  generic per-contributor experience fragment (excluding header/footer) instead
  of the hardcoded --stacey-roswells class, and list all 5 articles
- cards-byline parser: resolve the social network from href, link/aria text, or
  button icon class (these pages use href="#", so href-only matching missed all
  three links)
- add urls-magazine-articles.txt for the 4 re-migrated pages
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-skateparks.report.xlsx
+++ b/tools/importer/reports/import-skateparks.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="209">
   <si>
     <t>_reportFile</t>
   </si>
@@ -574,16 +574,13 @@
     <t>us/en/magazine/arctic-surfing.report.json</t>
   </si>
   <si>
-    <t>["breadcrumb"]</t>
-  </si>
-  <si>
     <t>us/en/magazine/arctic-surfing</t>
   </si>
   <si>
     <t>magazine-article</t>
   </si>
   <si>
-    <t>2026-09-14T20:18:50.537Z</t>
+    <t>2026-09-21T01:37:01.549Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -616,7 +613,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-09-14T20:19:00.328Z</t>
+    <t>2026-09-21T01:37:06.650Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -631,7 +628,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-09-14T20:19:04.728Z</t>
+    <t>2026-09-21T01:37:12.865Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -646,7 +643,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-09-14T20:19:09.061Z</t>
+    <t>2026-09-21T01:37:17.862Z</t>
   </si>
   <si>
     <t>Western Australia</t>
@@ -2272,159 +2269,159 @@
         <v>182</v>
       </c>
       <c r="B39" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" t="s">
+        <v>12</v>
+      </c>
+      <c r="D39" t="s">
+        <v>12</v>
+      </c>
+      <c r="E39" t="s">
         <v>183</v>
       </c>
-      <c r="C39" t="s">
-        <v>12</v>
-      </c>
-      <c r="D39" t="s">
-        <v>12</v>
-      </c>
-      <c r="E39" t="s">
+      <c r="F39" t="s">
+        <v>14</v>
+      </c>
+      <c r="G39" t="s">
         <v>184</v>
       </c>
-      <c r="F39" t="s">
-        <v>14</v>
-      </c>
-      <c r="G39" t="s">
+      <c r="H39" t="s">
         <v>185</v>
       </c>
-      <c r="H39" t="s">
+      <c r="I39" t="s">
         <v>186</v>
       </c>
-      <c r="I39" t="s">
+      <c r="J39" t="s">
         <v>187</v>
-      </c>
-      <c r="J39" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>188</v>
+      </c>
+      <c r="B40" t="s">
+        <v>12</v>
+      </c>
+      <c r="C40" t="s">
+        <v>12</v>
+      </c>
+      <c r="D40" t="s">
+        <v>12</v>
+      </c>
+      <c r="E40" t="s">
         <v>189</v>
       </c>
-      <c r="B40" t="s">
-        <v>12</v>
-      </c>
-      <c r="C40" t="s">
-        <v>12</v>
-      </c>
-      <c r="D40" t="s">
-        <v>12</v>
-      </c>
-      <c r="E40" t="s">
+      <c r="F40" t="s">
+        <v>14</v>
+      </c>
+      <c r="G40" t="s">
         <v>190</v>
       </c>
-      <c r="F40" t="s">
-        <v>14</v>
-      </c>
-      <c r="G40" t="s">
+      <c r="H40" t="s">
         <v>191</v>
       </c>
-      <c r="H40" t="s">
+      <c r="I40" t="s">
         <v>192</v>
       </c>
-      <c r="I40" t="s">
+      <c r="J40" t="s">
         <v>193</v>
-      </c>
-      <c r="J40" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>194</v>
+      </c>
+      <c r="B41" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" t="s">
+        <v>12</v>
+      </c>
+      <c r="D41" t="s">
+        <v>12</v>
+      </c>
+      <c r="E41" t="s">
         <v>195</v>
       </c>
-      <c r="B41" t="s">
-        <v>183</v>
-      </c>
-      <c r="C41" t="s">
-        <v>12</v>
-      </c>
-      <c r="D41" t="s">
-        <v>12</v>
-      </c>
-      <c r="E41" t="s">
+      <c r="F41" t="s">
+        <v>14</v>
+      </c>
+      <c r="G41" t="s">
+        <v>184</v>
+      </c>
+      <c r="H41" t="s">
         <v>196</v>
       </c>
-      <c r="F41" t="s">
-        <v>14</v>
-      </c>
-      <c r="G41" t="s">
-        <v>185</v>
-      </c>
-      <c r="H41" t="s">
+      <c r="I41" t="s">
         <v>197</v>
       </c>
-      <c r="I41" t="s">
+      <c r="J41" t="s">
         <v>198</v>
-      </c>
-      <c r="J41" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>199</v>
+      </c>
+      <c r="B42" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" t="s">
+        <v>12</v>
+      </c>
+      <c r="D42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E42" t="s">
         <v>200</v>
       </c>
-      <c r="B42" t="s">
-        <v>183</v>
-      </c>
-      <c r="C42" t="s">
-        <v>12</v>
-      </c>
-      <c r="D42" t="s">
-        <v>12</v>
-      </c>
-      <c r="E42" t="s">
+      <c r="F42" t="s">
+        <v>14</v>
+      </c>
+      <c r="G42" t="s">
+        <v>184</v>
+      </c>
+      <c r="H42" t="s">
         <v>201</v>
       </c>
-      <c r="F42" t="s">
-        <v>14</v>
-      </c>
-      <c r="G42" t="s">
-        <v>185</v>
-      </c>
-      <c r="H42" t="s">
+      <c r="I42" t="s">
         <v>202</v>
       </c>
-      <c r="I42" t="s">
+      <c r="J42" t="s">
         <v>203</v>
-      </c>
-      <c r="J42" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>204</v>
+      </c>
+      <c r="B43" t="s">
+        <v>12</v>
+      </c>
+      <c r="C43" t="s">
+        <v>12</v>
+      </c>
+      <c r="D43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" t="s">
         <v>205</v>
       </c>
-      <c r="B43" t="s">
-        <v>183</v>
-      </c>
-      <c r="C43" t="s">
-        <v>12</v>
-      </c>
-      <c r="D43" t="s">
-        <v>12</v>
-      </c>
-      <c r="E43" t="s">
+      <c r="F43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G43" t="s">
+        <v>184</v>
+      </c>
+      <c r="H43" t="s">
         <v>206</v>
       </c>
-      <c r="F43" t="s">
-        <v>14</v>
-      </c>
-      <c r="G43" t="s">
-        <v>185</v>
-      </c>
-      <c r="H43" t="s">
+      <c r="I43" t="s">
         <v>207</v>
       </c>
-      <c r="I43" t="s">
+      <c r="J43" t="s">
         <v>208</v>
-      </c>
-      <c r="J43" t="s">
-        <v>209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(cards): working PDF download on LA Skateparks
The source download href is an AEM-author DAM path
(/content/dam/.../ultimateguidetolaskateparks.pdf.coredownload.pdf) that 404s
on EDS. Host the real PDF on the content bus and link to it so the download
works.

- cards-button parser: rewrite the coredownload DAM href to the hosted PDF path
  (/us/en/magazine/la-skateparks/ultimateguidetolaskateparks.pdf)
- cards.js: add a `download` attribute to the button so it saves the file
- PDF uploaded to Document Authoring at that path (served 200 application/pdf)

Verified: old path 404s, new path 200s; the button downloads the file.
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-skateparks.report.xlsx
+++ b/tools/importer/reports/import-skateparks.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="430" uniqueCount="208">
   <si>
     <t>_reportFile</t>
   </si>
@@ -124,7 +124,7 @@
     <t>faqs</t>
   </si>
   <si>
-    <t>2026-09-14T15:15:52.540Z</t>
+    <t>2026-09-21T10:56:18.390Z</t>
   </si>
   <si>
     <t>FAQs</t>
@@ -595,10 +595,7 @@
     <t>us/en/magazine/guide-la-skateparks</t>
   </si>
   <si>
-    <t>skateparks-article</t>
-  </si>
-  <si>
-    <t>2026-09-21T00:41:38.123Z</t>
+    <t>2026-09-21T11:33:42.355Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -2316,33 +2313,33 @@
         <v>14</v>
       </c>
       <c r="G40" t="s">
+        <v>184</v>
+      </c>
+      <c r="H40" t="s">
         <v>190</v>
       </c>
-      <c r="H40" t="s">
+      <c r="I40" t="s">
         <v>191</v>
       </c>
-      <c r="I40" t="s">
+      <c r="J40" t="s">
         <v>192</v>
-      </c>
-      <c r="J40" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>193</v>
+      </c>
+      <c r="B41" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" t="s">
+        <v>12</v>
+      </c>
+      <c r="D41" t="s">
+        <v>12</v>
+      </c>
+      <c r="E41" t="s">
         <v>194</v>
-      </c>
-      <c r="B41" t="s">
-        <v>12</v>
-      </c>
-      <c r="C41" t="s">
-        <v>12</v>
-      </c>
-      <c r="D41" t="s">
-        <v>12</v>
-      </c>
-      <c r="E41" t="s">
-        <v>195</v>
       </c>
       <c r="F41" t="s">
         <v>14</v>
@@ -2351,30 +2348,30 @@
         <v>184</v>
       </c>
       <c r="H41" t="s">
+        <v>195</v>
+      </c>
+      <c r="I41" t="s">
         <v>196</v>
       </c>
-      <c r="I41" t="s">
+      <c r="J41" t="s">
         <v>197</v>
-      </c>
-      <c r="J41" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
+        <v>198</v>
+      </c>
+      <c r="B42" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" t="s">
+        <v>12</v>
+      </c>
+      <c r="D42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E42" t="s">
         <v>199</v>
-      </c>
-      <c r="B42" t="s">
-        <v>12</v>
-      </c>
-      <c r="C42" t="s">
-        <v>12</v>
-      </c>
-      <c r="D42" t="s">
-        <v>12</v>
-      </c>
-      <c r="E42" t="s">
-        <v>200</v>
       </c>
       <c r="F42" t="s">
         <v>14</v>
@@ -2383,30 +2380,30 @@
         <v>184</v>
       </c>
       <c r="H42" t="s">
+        <v>200</v>
+      </c>
+      <c r="I42" t="s">
         <v>201</v>
       </c>
-      <c r="I42" t="s">
+      <c r="J42" t="s">
         <v>202</v>
-      </c>
-      <c r="J42" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>203</v>
+      </c>
+      <c r="B43" t="s">
+        <v>12</v>
+      </c>
+      <c r="C43" t="s">
+        <v>12</v>
+      </c>
+      <c r="D43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" t="s">
         <v>204</v>
-      </c>
-      <c r="B43" t="s">
-        <v>12</v>
-      </c>
-      <c r="C43" t="s">
-        <v>12</v>
-      </c>
-      <c r="D43" t="s">
-        <v>12</v>
-      </c>
-      <c r="E43" t="s">
-        <v>205</v>
       </c>
       <c r="F43" t="s">
         <v>14</v>
@@ -2415,13 +2412,13 @@
         <v>184</v>
       </c>
       <c r="H43" t="s">
+        <v>205</v>
+      </c>
+      <c r="I43" t="s">
         <v>206</v>
       </c>
-      <c r="I43" t="s">
+      <c r="J43" t="s">
         <v>207</v>
-      </c>
-      <c r="J43" t="s">
-        <v>208</v>
       </c>
     </row>
   </sheetData>

</xml_diff>